<commit_message>
Replace real VINs, plates and battery codes with made-up test data
Examples, the practice eNEWS sample sheet, the template and the tests
had been filled with values copied from the dealer's screenshots, and
this repository is public. They are now obviously fake (TESTA…,
AAA001, TST01-1T1T01-T0001), and the default Excel path no longer
contains the user's name.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L35zGwhvYpwjtCuQ4cV3un
</commit_message>
<xml_diff>
--- a/enews_robotas/sablonas.xlsx
+++ b/enews_robotas/sablonas.xlsx
@@ -3239,22 +3239,22 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SJNJ12TD0U2373741</t>
+          <t>TESTA000000000002</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>JRH36</t>
+          <t>TST02</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>1Q9D77</t>
+          <t>1T2T02</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>TE204</t>
+          <t>T0002</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -3269,29 +3269,29 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>OAU289</t>
+          <t>AAA002</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>SJNJ12TD5U2387571</t>
+          <t>TESTA000000000003</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>JRJ36</t>
+          <t>TST01</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>1Q1H77</t>
+          <t>1T1T01</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>S3604</t>
+          <t>T0001</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -3306,7 +3306,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>AYT599</t>
+          <t>AAA003</t>
         </is>
       </c>
     </row>

</xml_diff>